<commit_message>
Corrige Corte 2: esquema TO-BE, ArchiMate y matrices verificadas
</commit_message>
<xml_diff>
--- a/05-seguridad-stride/tabla-stride-cliente.xlsx
+++ b/05-seguridad-stride/tabla-stride-cliente.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STRIDE" sheetId="1" r:id="R4c651261d16f4165"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STRIDE" sheetId="1" r:id="Re8a1adc829e64bd4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -141,7 +141,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -228,18 +228,27 @@
     <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="15">
+  <x:dxfs count="16">
     <x:dxf>
       <x:font>
         <x:b/>
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -250,7 +259,7 @@
         <x:color rgb="FF9C5700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE5CD"/>
         </x:patternFill>
       </x:fill>
@@ -261,7 +270,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -272,7 +281,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -283,7 +292,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -294,7 +303,7 @@
         <x:color rgb="FF9C5700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE5CD"/>
         </x:patternFill>
       </x:fill>
@@ -305,7 +314,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -316,7 +325,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -327,7 +336,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -338,7 +347,7 @@
         <x:color rgb="FF9C5700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE5CD"/>
         </x:patternFill>
       </x:fill>
@@ -349,7 +358,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -360,7 +369,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -371,7 +380,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -382,7 +391,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -392,8 +401,19 @@
         <x:color rgb="FF666666"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -419,10 +439,10 @@
     <x:tableColumn id="12" name="Nivel inherente"/>
     <x:tableColumn id="13" name="Estado del control"/>
     <x:tableColumn id="14" name="Responsable"/>
-    <x:tableColumn id="15" name="Probabilidad residual (1-5)"/>
-    <x:tableColumn id="16" name="Impacto residual (1-5)"/>
-    <x:tableColumn id="17" name="Puntaje residual"/>
-    <x:tableColumn id="18" name="Nivel residual"/>
+    <x:tableColumn id="15" name="P. residual proyectada (1–5)"/>
+    <x:tableColumn id="16" name="I. residual proyectado (1–5)"/>
+    <x:tableColumn id="17" name="Puntaje residual proyectado"/>
+    <x:tableColumn id="18" name="Nivel residual proyectado"/>
     <x:tableColumn id="19" name="Evidencia / validación"/>
     <x:tableColumn id="20" name="Tratamiento"/>
   </x:tableColumns>
@@ -698,7 +718,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="8" t="str">
-        <x:v>Evaluación preliminar del escenario objetivo. Los controles, responsables, probabilidades y evidencias deben validarse con Tecnología, Seguridad y la dueña del proceso antes de cerrar el diseño.</x:v>
+        <x:v>Evaluación inicial por validar. Riesgo residual PROYECTADO, condicionado a implantar y probar controles; no es riesgo observado. Criterios y fundamentos: criterios-priorizacion.md.</x:v>
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
@@ -720,7 +740,7 @@
       <x:c r="S3" s="8"/>
       <x:c r="T3" s="8"/>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="13" t="str">
         <x:v>Amenazas</x:v>
       </x:c>
@@ -734,21 +754,21 @@
       </x:c>
       <x:c r="E4" s="15" t="n">
         <x:f>COUNTIF(L9:L27,"Alto")+COUNTIF(L9:L27,"Crítico")</x:f>
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F4" s="2" t="str"/>
-      <x:c r="G4" s="13" t="str">
-        <x:v>Residual alto/crítico</x:v>
-      </x:c>
-      <x:c r="H4" s="15" t="n">
+      <x:c r="G4" s="30" t="str">
+        <x:v>Residual proyectado alto/crítico</x:v>
+      </x:c>
+      <x:c r="H4" s="31" t="n">
         <x:f>COUNTIF(R9:R27,"Alto")+COUNTIF(R9:R27,"Crítico")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="I4" s="16" t="str"/>
-      <x:c r="J4" s="17" t="str">
+      <x:c r="J4" s="32" t="str">
         <x:v>Controles por validar</x:v>
       </x:c>
-      <x:c r="K4" s="15" t="n">
+      <x:c r="K4" s="31" t="n">
         <x:f>COUNTIF(M9:M27,"Por validar")</x:f>
         <x:v>8</x:v>
       </x:c>
@@ -828,7 +848,7 @@
       <x:c r="S7" s="2"/>
       <x:c r="T7" s="2"/>
     </x:row>
-    <x:row r="8" ht="42" customHeight="1">
+    <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" s="21" t="str">
         <x:v>ID</x:v>
       </x:c>
@@ -872,16 +892,16 @@
         <x:v>Responsable</x:v>
       </x:c>
       <x:c r="O8" s="21" t="str">
-        <x:v>Probabilidad residual (1-5)</x:v>
+        <x:v>P. residual proyectada (1–5)</x:v>
       </x:c>
       <x:c r="P8" s="21" t="str">
-        <x:v>Impacto residual (1-5)</x:v>
+        <x:v>I. residual proyectado (1–5)</x:v>
       </x:c>
       <x:c r="Q8" s="21" t="str">
-        <x:v>Puntaje residual</x:v>
+        <x:v>Puntaje residual proyectado</x:v>
       </x:c>
       <x:c r="R8" s="21" t="str">
-        <x:v>Nivel residual</x:v>
+        <x:v>Nivel residual proyectado</x:v>
       </x:c>
       <x:c r="S8" s="21" t="str">
         <x:v>Evidencia / validación</x:v>
@@ -1484,7 +1504,7 @@
         <x:v>Mitigar</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="58" customHeight="1">
+    <x:row r="18" ht="112" customHeight="1">
       <x:c r="A18" s="24" t="str">
         <x:v>I-02</x:v>
       </x:c>
@@ -1544,13 +1564,13 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="S18" s="24" t="str">
-        <x:v>Reporte de accesos y revisión de grupos</x:v>
+        <x:v>I-02 residual proyectado 10 (Alto): revisar permisos efectivos y acordar tratamiento con Seguridad antes de datos reales. No aceptado.</x:v>
       </x:c>
       <x:c r="T18" s="24" t="str">
         <x:v>Mitigar</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="58" customHeight="1">
+    <x:row r="19" ht="112" customHeight="1">
       <x:c r="A19" s="24" t="str">
         <x:v>I-03</x:v>
       </x:c>
@@ -1570,10 +1590,10 @@
         <x:v>Divulgación pública, incidente de privacidad y afectación reputacional.</x:v>
       </x:c>
       <x:c r="G19" s="24" t="str">
-        <x:v>README declara uso de datos ficticios.</x:v>
+        <x:v>Regla de datos ficticios documentada y .gitignore incorporado al repositorio.</x:v>
       </x:c>
       <x:c r="H19" s="24" t="str">
-        <x:v>Regla de datos sintéticos, revisión antes de commit y exclusiones en .gitignore.</x:v>
+        <x:v>Revisión de archivos, capturas y metadatos antes de cada publicación. .gitignore no retira datos ya versionados ni detecta todo dato personal.</x:v>
       </x:c>
       <x:c r="I19" s="25" t="n">
         <x:v>3</x:v>
@@ -1590,7 +1610,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="M19" s="25" t="str">
-        <x:v>Existe</x:v>
+        <x:v>Parcial</x:v>
       </x:c>
       <x:c r="N19" s="25" t="str">
         <x:v>Equipo del proyecto</x:v>
@@ -1610,7 +1630,7 @@
         <x:v>Medio</x:v>
       </x:c>
       <x:c r="S19" s="24" t="str">
-        <x:v>Revisión del repositorio y checklist de publicación</x:v>
+        <x:v>README, .gitignore y checklist de publicación en informe.md; verificar cada nuevo commit.</x:v>
       </x:c>
       <x:c r="T19" s="24" t="str">
         <x:v>Mitigar</x:v>
@@ -1748,7 +1768,7 @@
         <x:v>Mitigar</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="58" customHeight="1">
+    <x:row r="22" ht="98" customHeight="1">
       <x:c r="A22" s="24" t="str">
         <x:v>D-02</x:v>
       </x:c>
@@ -1774,14 +1794,14 @@
         <x:v>Plantilla de entrada, validación de esquema, mensaje de error y manejo de excepciones.</x:v>
       </x:c>
       <x:c r="I22" s="25" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J22" s="25" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="K22" s="26" t="n">
         <x:f>I22*J22</x:f>
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="L22" s="25" t="str">
         <x:f>IF(K22&gt;=17,"Crítico",IF(K22&gt;=10,"Alto",IF(K22&gt;=5,"Medio","Bajo")))</x:f>
@@ -1808,7 +1828,7 @@
         <x:v>Medio</x:v>
       </x:c>
       <x:c r="S22" s="24" t="str">
-        <x:v>Caso de prueba con esquema inválido</x:v>
+        <x:v>Prueba de cambio de esquema; probabilidad 3 por falta de recurrencia documentada. Ver criterios-priorizacion.md.</x:v>
       </x:c>
       <x:c r="T22" s="24" t="str">
         <x:v>Mitigar</x:v>
@@ -1880,7 +1900,7 @@
         <x:v>Mitigar</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="58" customHeight="1">
+    <x:row r="24" ht="98" customHeight="1">
       <x:c r="A24" s="24" t="str">
         <x:v>D-04</x:v>
       </x:c>
@@ -1906,18 +1926,18 @@
         <x:v>Calendario, responsable suplente, alerta de ausencia y escalamiento.</x:v>
       </x:c>
       <x:c r="I24" s="25" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J24" s="25" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="K24" s="26" t="n">
         <x:f>I24*J24</x:f>
-        <x:v>12</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="L24" s="25" t="str">
         <x:f>IF(K24&gt;=17,"Crítico",IF(K24&gt;=10,"Alto",IF(K24&gt;=5,"Medio","Bajo")))</x:f>
-        <x:v>Alto</x:v>
+        <x:v>Medio</x:v>
       </x:c>
       <x:c r="M24" s="25" t="str">
         <x:v>Propuesto</x:v>
@@ -1940,7 +1960,7 @@
         <x:v>Bajo</x:v>
       </x:c>
       <x:c r="S24" s="24" t="str">
-        <x:v>Calendario y prueba de alerta</x:v>
+        <x:v>Validar calendario y latencia; probabilidad 2, sin evidencia de bloqueos recurrentes. Ver criterios-priorizacion.md.</x:v>
       </x:c>
       <x:c r="T24" s="24" t="str">
         <x:v>Mitigar</x:v>
@@ -2190,7 +2210,7 @@
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
       <x:c r="A30" s="29" t="str">
-        <x:v>Fuentes principales: Microsoft Learn (permisos de SharePoint, conectores/DLP y aprobaciones de Power Automate) y OWASP Threat Modeling. Véase referencias.md en esta carpeta.</x:v>
+        <x:v>Fuentes: Microsoft Learn y referencias.md. Escalas, fundamentos por amenaza y cambios D-02/D-04: criterios-priorizacion.md. I-02 conserva riesgo residual proyectado Alto y tratamiento pendiente de aprobación.</x:v>
       </x:c>
       <x:c r="B30" s="29"/>
       <x:c r="C30" s="29"/>
@@ -2898,6 +2918,7 @@
     <x:cfRule type="containsText" dxfId="12" priority="13" operator="containsText" text="Existe"/>
     <x:cfRule type="containsText" dxfId="13" priority="14" operator="containsText" text="Cumple"/>
     <x:cfRule type="containsText" dxfId="14" priority="15" operator="containsText" text="No aplica"/>
+    <x:cfRule type="containsText" dxfId="15" priority="16" operator="containsText" text="Parcial"/>
   </x:conditionalFormatting>
   <x:dataValidations count="7">
     <x:dataValidation type="list" sqref="B9:B27">
@@ -2920,7 +2941,7 @@
       <x:formula2>5</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="M9:M27">
-      <x:formula1>"Existe,Propuesto,Por validar"</x:formula1>
+      <x:formula1>"Existe,Parcial,Propuesto,Por validar"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="T9:T27">
       <x:formula1>"Mitigar,Aceptar,Transferir,Evitar"</x:formula1>
@@ -2928,7 +2949,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb0e3d4b328a4f38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra34f2f830bb8491a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>